<commit_message>
Excel: backfill 6 seed signals into Signals sheet (HSCL/ASTERDM + 4 no_fill)
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -21,13 +21,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,86 +547,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Signal_Date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Prev_Close</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>SL</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Range_Pct</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Close_Pos</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Volume_Spike</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Below_VWAP</t>
         </is>
@@ -679,6 +691,274 @@
       <c r="P2" t="b">
         <v>1</v>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>11:30:20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>704.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>698.5700000000001</v>
+      </c>
+      <c r="H3" t="n">
+        <v>681.1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>706.95</v>
+      </c>
+      <c r="J3" t="n">
+        <v>718.13</v>
+      </c>
+      <c r="K3" t="n">
+        <v>10.37</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="M3" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>11:30:20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>765.65</v>
+      </c>
+      <c r="G4" t="n">
+        <v>759.52</v>
+      </c>
+      <c r="H4" t="n">
+        <v>740.54</v>
+      </c>
+      <c r="I4" t="n">
+        <v>768.64</v>
+      </c>
+      <c r="J4" t="n">
+        <v>780.79</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="M4" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>11:30:20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>NO_FILL (no_fill)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>11:30:20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NO_FILL (no_fill)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>11:30:20</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>JSWCEMENT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NO_FILL (no_fill)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11:30:20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SOBHA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NO_FILL (no_fill)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Prod: broker-type simulator, full TG events, 15-min live git auto
- executor.py: BrokerSimulator class (ENTRY LIMIT/SL-M/T1/T2/MARKET orders,
  lifecycle PLACED->FILLED/CANCELLED/REJECTED, close-based exits,
  OPEN positions monitored across runs, T1 books 50% + SL->BE)
- portfolio.py: holdings/orders/daily_pnl schema, can_take_trade per date
- telegram_notifier.py: emoji event messages + summary + doc, retry x3
- excel_logger.py: Orders sheet added to existing files
- main.py: LIVE_MODE intraday processing, holding monitor, TG events
- workflow: cron */15 3-10 * * 1-5 (08:30-16:29 IST), LIVE_MODE=1
- live_auto.ps1: local loop equivalent
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,66 +430,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Stocks_Scanned</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Daily_Ok</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Intraday_Ok</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Signals_Found</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Tradeable</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Watchlist</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Errors</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Duration_Sec</t>
         </is>
@@ -534,6 +535,90 @@
       </c>
       <c r="L2" t="n">
         <v>39.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12:35:21</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>500</v>
+      </c>
+      <c r="D3" t="n">
+        <v>500</v>
+      </c>
+      <c r="E3" t="n">
+        <v>500</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>47.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12:37:11</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>500</v>
+      </c>
+      <c r="D4" t="n">
+        <v>500</v>
+      </c>
+      <c r="E4" t="n">
+        <v>500</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>43.6</v>
       </c>
     </row>
   </sheetData>
@@ -742,7 +827,6 @@
       <c r="M3" t="n">
         <v>36.7</v>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="b">
         <v>1</v>
       </c>
@@ -800,7 +884,6 @@
       <c r="M4" t="n">
         <v>32.9</v>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="b">
         <v>1</v>
       </c>
@@ -834,17 +917,6 @@
           <t>NO_FILL (no_fill)</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -872,17 +944,6 @@
           <t>NO_FILL (no_fill)</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -910,17 +971,6 @@
           <t>NO_FILL (no_fill)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -948,17 +998,6 @@
           <t>NO_FILL (no_fill)</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1103,61 +1142,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Capital</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unrealized_PnL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Total_PnL</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Win_Rate</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
@@ -1200,6 +1239,731 @@
       </c>
       <c r="K2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>19653.74</v>
+      </c>
+      <c r="E3" t="n">
+        <v>180346.26</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12:37:11</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>19653.74</v>
+      </c>
+      <c r="E4" t="n">
+        <v>180346.26</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Order_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12:35:21</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>47BA4CE1D8</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>698.5700000000001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12:35:21</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>47BA4CE1D8</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>698.5700000000001</v>
+      </c>
+      <c r="I3" t="n">
+        <v>14</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>@ 2026-08-21 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12:35:21</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>5EA6E49CEA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>681.1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>14</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3801A9DCAF</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>706.95</v>
+      </c>
+      <c r="I5" t="n">
+        <v>7</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8771967073</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>718.13</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A7F19BF582</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>759.52</v>
+      </c>
+      <c r="I7" t="n">
+        <v>13</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A7F19BF582</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>759.52</v>
+      </c>
+      <c r="I8" t="n">
+        <v>13</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>@ 2026-08-21 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AA566CF22F</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>740.54</v>
+      </c>
+      <c r="I9" t="n">
+        <v>13</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>24AAEC949E</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>768.64</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>30A84F839F</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>780.79</v>
+      </c>
+      <c r="I11" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>C7A089A400</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PFOCUS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>276.97</v>
+      </c>
+      <c r="I12" t="n">
+        <v>36</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12:35:22</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>C7A089A400</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PFOCUS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>276.97</v>
+      </c>
+      <c r="I13" t="n">
+        <v>36</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
state: bot run 2026-08-21T12:38 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,6 +619,48 @@
       </c>
       <c r="L4" t="n">
         <v>43.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12:38:55</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>500</v>
+      </c>
+      <c r="D5" t="n">
+        <v>500</v>
+      </c>
+      <c r="E5" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>34.6</v>
       </c>
     </row>
   </sheetData>
@@ -1142,7 +1184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1316,6 +1358,45 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12:38:55</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19653.74</v>
+      </c>
+      <c r="E5" t="n">
+        <v>180346.26</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-21T13:30 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -661,6 +661,48 @@
       </c>
       <c r="L5" t="n">
         <v>34.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>13:30:12</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>500</v>
+      </c>
+      <c r="D6" t="n">
+        <v>500</v>
+      </c>
+      <c r="E6" t="n">
+        <v>500</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>36.8</v>
       </c>
     </row>
   </sheetData>
@@ -1184,7 +1226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1397,6 +1439,45 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>13:30:12</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>19653.74</v>
+      </c>
+      <c r="E6" t="n">
+        <v>180346.26</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-21T14:24 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -703,6 +703,48 @@
       </c>
       <c r="L6" t="n">
         <v>36.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>14:24:10</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>500</v>
+      </c>
+      <c r="E7" t="n">
+        <v>500</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>39.2</v>
       </c>
     </row>
   </sheetData>
@@ -716,7 +758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -854,10 +896,10 @@
       <c r="N2" t="n">
         <v>286.31</v>
       </c>
-      <c r="O2" t="b">
+      <c r="O2" t="n">
         <v>1</v>
       </c>
-      <c r="P2" t="b">
+      <c r="P2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -911,10 +953,10 @@
       <c r="M3" t="n">
         <v>36.7</v>
       </c>
-      <c r="O3" t="b">
+      <c r="O3" t="n">
         <v>1</v>
       </c>
-      <c r="P3" t="b">
+      <c r="P3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -968,10 +1010,10 @@
       <c r="M4" t="n">
         <v>32.9</v>
       </c>
-      <c r="O4" t="b">
+      <c r="O4" t="n">
         <v>1</v>
       </c>
-      <c r="P4" t="b">
+      <c r="P4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1081,6 +1123,66 @@
         <is>
           <t>NO_FILL (no_fill)</t>
         </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>14:24:10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CROMPTON</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>251.25</v>
+      </c>
+      <c r="G9" t="n">
+        <v>249.24</v>
+      </c>
+      <c r="H9" t="n">
+        <v>243.01</v>
+      </c>
+      <c r="I9" t="n">
+        <v>252.23</v>
+      </c>
+      <c r="J9" t="n">
+        <v>256.22</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="M9" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="N9" t="n">
+        <v>253.7</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1226,7 +1328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1478,6 +1580,45 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>14:24:10</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>19653.74</v>
+      </c>
+      <c r="E7" t="n">
+        <v>180346.26</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-21T15:14 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -745,6 +745,48 @@
       </c>
       <c r="L7" t="n">
         <v>39.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>15:14:05</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>500</v>
+      </c>
+      <c r="D8" t="n">
+        <v>500</v>
+      </c>
+      <c r="E8" t="n">
+        <v>500</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>38.3</v>
       </c>
     </row>
   </sheetData>
@@ -758,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1182,6 +1224,126 @@
         <v>1</v>
       </c>
       <c r="P9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15:14:05</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1082.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1073.44</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1046.61</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1086.32</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1103.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="M10" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1140.24</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:14:05</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>655.25</v>
+      </c>
+      <c r="G11" t="n">
+        <v>650.01</v>
+      </c>
+      <c r="H11" t="n">
+        <v>633.76</v>
+      </c>
+      <c r="I11" t="n">
+        <v>657.8099999999999</v>
+      </c>
+      <c r="J11" t="n">
+        <v>668.21</v>
+      </c>
+      <c r="K11" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="M11" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="N11" t="n">
+        <v>755.71</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1196,7 +1358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1273,6 +1435,63 @@
       <c r="O1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>698.5700000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F2" t="n">
+        <v>681.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>706.95</v>
+      </c>
+      <c r="H2" t="n">
+        <v>718.13</v>
+      </c>
+      <c r="I2" t="n">
+        <v>681.1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>-2.501</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-2.801</v>
+      </c>
+      <c r="M2" t="n">
+        <v>9779.98</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-273.94</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1620,6 +1839,45 @@
       </c>
       <c r="K7" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>15:14:05</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>199726.06</v>
+      </c>
+      <c r="D8" t="n">
+        <v>9873.76</v>
+      </c>
+      <c r="E8" t="n">
+        <v>189852.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1633,7 +1891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2269,6 +2527,54 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>15:14:05</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>104B9E10B8</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>681.1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>14</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>STOP_LOSS close 663.70 low 662.40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-08-21T15:45 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -787,6 +787,48 @@
       </c>
       <c r="L8" t="n">
         <v>38.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15:45:13</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>500</v>
+      </c>
+      <c r="D9" t="n">
+        <v>500</v>
+      </c>
+      <c r="E9" t="n">
+        <v>500</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>44.8</v>
       </c>
     </row>
   </sheetData>
@@ -1358,7 +1400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1490,6 +1532,63 @@
         <v>-273.94</v>
       </c>
       <c r="O2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>759.52</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F3" t="n">
+        <v>740.54</v>
+      </c>
+      <c r="G3" t="n">
+        <v>768.64</v>
+      </c>
+      <c r="H3" t="n">
+        <v>780.79</v>
+      </c>
+      <c r="I3" t="n">
+        <v>761.35</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-0.059</v>
+      </c>
+      <c r="M3" t="n">
+        <v>9873.76</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -1547,7 +1646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1878,6 +1977,45 @@
       </c>
       <c r="K8" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15:45:13</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1891,7 +2029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2575,6 +2713,51 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15:45:13</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3200739B29</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>13</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>time exit @ 761.35</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-08-21T16:23 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -829,6 +829,48 @@
       </c>
       <c r="L9" t="n">
         <v>44.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>16:23:11</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>500</v>
+      </c>
+      <c r="D10" t="n">
+        <v>500</v>
+      </c>
+      <c r="E10" t="n">
+        <v>500</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>28.7</v>
       </c>
     </row>
   </sheetData>
@@ -1646,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2015,6 +2057,45 @@
         <v>2</v>
       </c>
       <c r="K9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>16:23:11</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T09:30 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -871,6 +871,48 @@
       </c>
       <c r="L10" t="n">
         <v>28.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:30:09</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>500</v>
+      </c>
+      <c r="D11" t="n">
+        <v>500</v>
+      </c>
+      <c r="E11" t="n">
+        <v>500</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1688,7 +1730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2096,6 +2138,45 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:30:09</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T10:27 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -913,6 +913,48 @@
       </c>
       <c r="L11" t="n">
         <v>30</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:27:19</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D12" t="n">
+        <v>500</v>
+      </c>
+      <c r="E12" t="n">
+        <v>500</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>32.8</v>
       </c>
     </row>
   </sheetData>
@@ -1730,7 +1772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2177,6 +2219,45 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:27:19</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T11:17 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -955,6 +955,48 @@
       </c>
       <c r="L12" t="n">
         <v>32.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:17:17</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>500</v>
+      </c>
+      <c r="D13" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" t="n">
+        <v>500</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>27.6</v>
       </c>
     </row>
   </sheetData>
@@ -1772,7 +1814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2258,6 +2300,45 @@
         <v>2</v>
       </c>
       <c r="K12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:17:17</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T12:41 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -997,6 +997,48 @@
       </c>
       <c r="L13" t="n">
         <v>27.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12:41:27</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>500</v>
+      </c>
+      <c r="D14" t="n">
+        <v>500</v>
+      </c>
+      <c r="E14" t="n">
+        <v>500</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>38.2</v>
       </c>
     </row>
   </sheetData>
@@ -1814,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2339,6 +2381,45 @@
         <v>2</v>
       </c>
       <c r="K13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12:41:27</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T13:36 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1039,6 +1039,48 @@
       </c>
       <c r="L14" t="n">
         <v>38.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:36:55</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>500</v>
+      </c>
+      <c r="D15" t="n">
+        <v>500</v>
+      </c>
+      <c r="E15" t="n">
+        <v>500</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>37.6</v>
       </c>
     </row>
   </sheetData>
@@ -1856,7 +1898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2420,6 +2462,45 @@
         <v>2</v>
       </c>
       <c r="K14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:36:56</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T14:37 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,6 +1081,48 @@
       </c>
       <c r="L15" t="n">
         <v>37.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>500</v>
+      </c>
+      <c r="D16" t="n">
+        <v>500</v>
+      </c>
+      <c r="E16" t="n">
+        <v>500</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>30.1</v>
       </c>
     </row>
   </sheetData>
@@ -1094,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1638,6 +1680,126 @@
         <v>1</v>
       </c>
       <c r="P11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>COROMANDEL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1929.8</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1914.36</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1866.5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1937.33</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1967.96</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="M12" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2061.61</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CREDITACC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1443.7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1432.15</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1396.35</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1449.34</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1472.25</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="M13" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1542.63</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1898,7 +2060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2501,6 +2663,45 @@
         <v>2</v>
       </c>
       <c r="K15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:37:21</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T15:37 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1123,6 +1123,48 @@
       </c>
       <c r="L16" t="n">
         <v>30.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15:37:07</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>500</v>
+      </c>
+      <c r="D17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E17" t="n">
+        <v>500</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>39.6</v>
       </c>
     </row>
   </sheetData>
@@ -1136,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1800,6 +1842,126 @@
         <v>1</v>
       </c>
       <c r="P13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>15:37:07</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GODREJIND</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1184.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1175.02</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1145.65</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1189.12</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1207.92</v>
+      </c>
+      <c r="K14" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="M14" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1272.31</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15:37:07</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>HSCL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>662.2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>656.9</v>
+      </c>
+      <c r="H15" t="n">
+        <v>640.48</v>
+      </c>
+      <c r="I15" t="n">
+        <v>664.79</v>
+      </c>
+      <c r="J15" t="n">
+        <v>675.3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="M15" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="N15" t="n">
+        <v>749.25</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2060,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2702,6 +2864,45 @@
         <v>2</v>
       </c>
       <c r="K16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15:37:07</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-24T16:26 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1165,6 +1165,48 @@
       </c>
       <c r="L17" t="n">
         <v>39.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>16:26:32</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>500</v>
+      </c>
+      <c r="D18" t="n">
+        <v>500</v>
+      </c>
+      <c r="E18" t="n">
+        <v>500</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>43.7</v>
       </c>
     </row>
   </sheetData>
@@ -2222,7 +2264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2903,6 +2945,45 @@
         <v>2</v>
       </c>
       <c r="K17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>16:26:32</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T09:24 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1207,6 +1207,48 @@
       </c>
       <c r="L18" t="n">
         <v>43.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09:24:17</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>500</v>
+      </c>
+      <c r="D19" t="n">
+        <v>500</v>
+      </c>
+      <c r="E19" t="n">
+        <v>500</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>48.9</v>
       </c>
     </row>
   </sheetData>
@@ -2264,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2984,6 +3026,45 @@
         <v>2</v>
       </c>
       <c r="K18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09:24:17</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T10:17 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1249,6 +1249,48 @@
       </c>
       <c r="L19" t="n">
         <v>48.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:17:13</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>500</v>
+      </c>
+      <c r="D20" t="n">
+        <v>500</v>
+      </c>
+      <c r="E20" t="n">
+        <v>500</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>68.3</v>
       </c>
     </row>
   </sheetData>
@@ -2306,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3065,6 +3107,45 @@
         <v>2</v>
       </c>
       <c r="K19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:17:13</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T11:08 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,6 +1291,48 @@
       </c>
       <c r="L20" t="n">
         <v>68.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:08:29</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>500</v>
+      </c>
+      <c r="D21" t="n">
+        <v>500</v>
+      </c>
+      <c r="E21" t="n">
+        <v>500</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -2348,7 +2390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3146,6 +3188,45 @@
         <v>2</v>
       </c>
       <c r="K20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:08:29</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T11:47 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1333,6 +1333,48 @@
       </c>
       <c r="L21" t="n">
         <v>47</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:47:56</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>500</v>
+      </c>
+      <c r="D22" t="n">
+        <v>500</v>
+      </c>
+      <c r="E22" t="n">
+        <v>500</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>38.2</v>
       </c>
     </row>
   </sheetData>
@@ -1346,7 +1388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2130,6 +2172,66 @@
         <v>1</v>
       </c>
       <c r="P15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:47:56</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CHAMBLFERT</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>430.35</v>
+      </c>
+      <c r="G16" t="n">
+        <v>426.91</v>
+      </c>
+      <c r="H16" t="n">
+        <v>416.23</v>
+      </c>
+      <c r="I16" t="n">
+        <v>432.03</v>
+      </c>
+      <c r="J16" t="n">
+        <v>438.86</v>
+      </c>
+      <c r="K16" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="M16" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="N16" t="n">
+        <v>441.07</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2390,7 +2492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3227,6 +3329,45 @@
         <v>2</v>
       </c>
       <c r="K21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:47:56</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T12:57 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1375,6 +1375,48 @@
       </c>
       <c r="L22" t="n">
         <v>38.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:57:14</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>500</v>
+      </c>
+      <c r="D23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E23" t="n">
+        <v>500</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>41.7</v>
       </c>
     </row>
   </sheetData>
@@ -1388,7 +1430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2232,6 +2274,66 @@
         <v>1</v>
       </c>
       <c r="P16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12:57:14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>RAMCOCEM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>904.75</v>
+      </c>
+      <c r="G17" t="n">
+        <v>897.51</v>
+      </c>
+      <c r="H17" t="n">
+        <v>875.0700000000001</v>
+      </c>
+      <c r="I17" t="n">
+        <v>908.28</v>
+      </c>
+      <c r="J17" t="n">
+        <v>922.64</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="M17" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="N17" t="n">
+        <v>919.24</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2492,7 +2594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3368,6 +3470,45 @@
         <v>2</v>
       </c>
       <c r="K22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:57:14</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T13:41 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1417,6 +1417,48 @@
       </c>
       <c r="L23" t="n">
         <v>41.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:41:37</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>500</v>
+      </c>
+      <c r="D24" t="n">
+        <v>500</v>
+      </c>
+      <c r="E24" t="n">
+        <v>500</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>45.9</v>
       </c>
     </row>
   </sheetData>
@@ -2594,7 +2636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3509,6 +3551,45 @@
         <v>2</v>
       </c>
       <c r="K23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:41:37</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T14:33 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1459,6 +1459,48 @@
       </c>
       <c r="L24" t="n">
         <v>45.9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:33:26</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>500</v>
+      </c>
+      <c r="D25" t="n">
+        <v>500</v>
+      </c>
+      <c r="E25" t="n">
+        <v>500</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>49.4</v>
       </c>
     </row>
   </sheetData>
@@ -2636,7 +2678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3590,6 +3632,45 @@
         <v>2</v>
       </c>
       <c r="K24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:33:26</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T15:23 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1501,6 +1501,48 @@
       </c>
       <c r="L25" t="n">
         <v>49.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:23:57</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>500</v>
+      </c>
+      <c r="D26" t="n">
+        <v>500</v>
+      </c>
+      <c r="E26" t="n">
+        <v>500</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>38.2</v>
       </c>
     </row>
   </sheetData>
@@ -2678,7 +2720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3671,6 +3713,45 @@
         <v>2</v>
       </c>
       <c r="K25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:23:57</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T16:10 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1543,6 +1543,48 @@
       </c>
       <c r="L26" t="n">
         <v>38.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>16:09:57</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>500</v>
+      </c>
+      <c r="D27" t="n">
+        <v>500</v>
+      </c>
+      <c r="E27" t="n">
+        <v>500</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>41.1</v>
       </c>
     </row>
   </sheetData>
@@ -2720,7 +2762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3752,6 +3794,45 @@
         <v>2</v>
       </c>
       <c r="K26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>16:09:57</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-25T16:41 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1585,6 +1585,48 @@
       </c>
       <c r="L27" t="n">
         <v>41.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:41:21</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>500</v>
+      </c>
+      <c r="D28" t="n">
+        <v>500</v>
+      </c>
+      <c r="E28" t="n">
+        <v>500</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>39.2</v>
       </c>
     </row>
   </sheetData>
@@ -2762,7 +2804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3833,6 +3875,45 @@
         <v>2</v>
       </c>
       <c r="K27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:41:21</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T09:28 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1627,6 +1627,48 @@
       </c>
       <c r="L28" t="n">
         <v>39.2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:28:48</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>500</v>
+      </c>
+      <c r="D29" t="n">
+        <v>500</v>
+      </c>
+      <c r="E29" t="n">
+        <v>500</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>47.4</v>
       </c>
     </row>
   </sheetData>
@@ -1640,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2544,6 +2586,66 @@
         <v>1</v>
       </c>
       <c r="P17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:28:48</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>428.6</v>
+      </c>
+      <c r="G18" t="n">
+        <v>425.17</v>
+      </c>
+      <c r="H18" t="n">
+        <v>414.54</v>
+      </c>
+      <c r="I18" t="n">
+        <v>430.27</v>
+      </c>
+      <c r="J18" t="n">
+        <v>437.08</v>
+      </c>
+      <c r="K18" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="M18" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="N18" t="n">
+        <v>438.33</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2804,7 +2906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3914,6 +4016,45 @@
         <v>2</v>
       </c>
       <c r="K28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:28:48</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T10:20 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1669,6 +1669,48 @@
       </c>
       <c r="L29" t="n">
         <v>47.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10:20:52</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>500</v>
+      </c>
+      <c r="D30" t="n">
+        <v>500</v>
+      </c>
+      <c r="E30" t="n">
+        <v>500</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>34.8</v>
       </c>
     </row>
   </sheetData>
@@ -2906,7 +2948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4055,6 +4097,45 @@
         <v>2</v>
       </c>
       <c r="K29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10:20:52</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T11:10 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1711,6 +1711,48 @@
       </c>
       <c r="L30" t="n">
         <v>34.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11:10:43</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>500</v>
+      </c>
+      <c r="D31" t="n">
+        <v>500</v>
+      </c>
+      <c r="E31" t="n">
+        <v>500</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -2948,7 +2990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4136,6 +4178,45 @@
         <v>2</v>
       </c>
       <c r="K30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11:10:43</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T11:50 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1753,6 +1753,48 @@
       </c>
       <c r="L31" t="n">
         <v>44</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11:50:44</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>500</v>
+      </c>
+      <c r="D32" t="n">
+        <v>500</v>
+      </c>
+      <c r="E32" t="n">
+        <v>500</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2990,7 +3032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4217,6 +4259,45 @@
         <v>2</v>
       </c>
       <c r="K31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11:50:44</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T12:58 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1795,6 +1795,48 @@
       </c>
       <c r="L32" t="n">
         <v>45</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:58:36</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>500</v>
+      </c>
+      <c r="D33" t="n">
+        <v>500</v>
+      </c>
+      <c r="E33" t="n">
+        <v>500</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>33.7</v>
       </c>
     </row>
   </sheetData>
@@ -3032,7 +3074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4298,6 +4340,45 @@
         <v>2</v>
       </c>
       <c r="K32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:58:36</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T13:51 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1837,6 +1837,48 @@
       </c>
       <c r="L33" t="n">
         <v>33.7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>13:51:24</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>500</v>
+      </c>
+      <c r="D34" t="n">
+        <v>500</v>
+      </c>
+      <c r="E34" t="n">
+        <v>500</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>44.4</v>
       </c>
     </row>
   </sheetData>
@@ -1850,7 +1892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2814,6 +2856,66 @@
         <v>1</v>
       </c>
       <c r="P18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:51:24</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PREMIERENE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>993.1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>985.16</v>
+      </c>
+      <c r="H19" t="n">
+        <v>960.53</v>
+      </c>
+      <c r="I19" t="n">
+        <v>996.98</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1012.74</v>
+      </c>
+      <c r="K19" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="M19" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1027.62</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3074,7 +3176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4379,6 +4481,45 @@
         <v>2</v>
       </c>
       <c r="K33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>13:51:24</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T14:51 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1879,6 +1879,48 @@
       </c>
       <c r="L34" t="n">
         <v>44.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14:51:00</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>500</v>
+      </c>
+      <c r="D35" t="n">
+        <v>500</v>
+      </c>
+      <c r="E35" t="n">
+        <v>500</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>32.2</v>
       </c>
     </row>
   </sheetData>
@@ -3176,7 +3218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4520,6 +4562,45 @@
         <v>2</v>
       </c>
       <c r="K34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14:51:00</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T15:38 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1921,6 +1921,48 @@
       </c>
       <c r="L35" t="n">
         <v>32.2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:38:19</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>500</v>
+      </c>
+      <c r="D36" t="n">
+        <v>500</v>
+      </c>
+      <c r="E36" t="n">
+        <v>500</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>45.7</v>
       </c>
     </row>
   </sheetData>
@@ -3218,7 +3260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4601,6 +4643,45 @@
         <v>2</v>
       </c>
       <c r="K35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:38:19</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-26T16:23 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1963,6 +1963,48 @@
       </c>
       <c r="L36" t="n">
         <v>45.7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:23:31</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>500</v>
+      </c>
+      <c r="D37" t="n">
+        <v>500</v>
+      </c>
+      <c r="E37" t="n">
+        <v>500</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>28.3</v>
       </c>
     </row>
   </sheetData>
@@ -3260,7 +3302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4682,6 +4724,45 @@
         <v>2</v>
       </c>
       <c r="K36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:23:31</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>199720.23</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-08-27T19:32 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2005,6 +2005,48 @@
       </c>
       <c r="L37" t="n">
         <v>28.3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:32:15</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>500</v>
+      </c>
+      <c r="D38" t="n">
+        <v>500</v>
+      </c>
+      <c r="E38" t="n">
+        <v>500</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>34.1</v>
       </c>
     </row>
   </sheetData>
@@ -2018,7 +2060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3042,6 +3084,126 @@
         <v>1</v>
       </c>
       <c r="P19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>611.9</v>
+      </c>
+      <c r="G20" t="n">
+        <v>607</v>
+      </c>
+      <c r="H20" t="n">
+        <v>591.83</v>
+      </c>
+      <c r="I20" t="n">
+        <v>614.29</v>
+      </c>
+      <c r="J20" t="n">
+        <v>624</v>
+      </c>
+      <c r="K20" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="M20" t="n">
+        <v>39</v>
+      </c>
+      <c r="N20" t="n">
+        <v>619.58</v>
+      </c>
+      <c r="O20" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>387.7</v>
+      </c>
+      <c r="G21" t="n">
+        <v>384.6</v>
+      </c>
+      <c r="H21" t="n">
+        <v>374.98</v>
+      </c>
+      <c r="I21" t="n">
+        <v>389.21</v>
+      </c>
+      <c r="J21" t="n">
+        <v>395.37</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="N21" t="n">
+        <v>402.36</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3056,7 +3218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3245,6 +3407,63 @@
         <v>-5.83</v>
       </c>
       <c r="O3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>425.17</v>
+      </c>
+      <c r="E4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F4" t="n">
+        <v>414.54</v>
+      </c>
+      <c r="G4" t="n">
+        <v>430.27</v>
+      </c>
+      <c r="H4" t="n">
+        <v>437.08</v>
+      </c>
+      <c r="I4" t="n">
+        <v>420</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>-1.216</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-1.516</v>
+      </c>
+      <c r="M4" t="n">
+        <v>9778.91</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-148.25</v>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -3302,7 +3521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4763,6 +4982,45 @@
         <v>2</v>
       </c>
       <c r="K37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>199571.98</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>199571.98</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-4.38</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-4.38</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4777,7 +5035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5506,6 +5764,339 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>70D53178A7</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>425.17</v>
+      </c>
+      <c r="I16" t="n">
+        <v>23</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>70D53178A7</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>425.17</v>
+      </c>
+      <c r="I17" t="n">
+        <v>23</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>@ 2026-08-27 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10813ADC49</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>414.54</v>
+      </c>
+      <c r="I18" t="n">
+        <v>23</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A448127CAF</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>430.27</v>
+      </c>
+      <c r="I19" t="n">
+        <v>11</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>D149656F76</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>437.08</v>
+      </c>
+      <c r="I20" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1208C0C09D</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>23</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>time exit @ 420.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>19:32:16</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AA8BE7B671</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PREMIERENE</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>985.16</v>
+      </c>
+      <c r="I22" t="n">
+        <v>10</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>gap-up open 1002.20 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-08-28T20:43 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2047,6 +2047,48 @@
       </c>
       <c r="L38" t="n">
         <v>34.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>500</v>
+      </c>
+      <c r="D39" t="n">
+        <v>500</v>
+      </c>
+      <c r="E39" t="n">
+        <v>500</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>37.7</v>
       </c>
     </row>
   </sheetData>
@@ -2060,7 +2102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3204,6 +3246,66 @@
         <v>1</v>
       </c>
       <c r="P21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1275.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1265.3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1233.66</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1280.48</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1300.72</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="M22" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1367.63</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3218,7 +3320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3464,6 +3566,63 @@
         <v>-148.25</v>
       </c>
       <c r="O4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>384.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>26</v>
+      </c>
+      <c r="F5" t="n">
+        <v>374.98</v>
+      </c>
+      <c r="G5" t="n">
+        <v>389.21</v>
+      </c>
+      <c r="H5" t="n">
+        <v>395.37</v>
+      </c>
+      <c r="I5" t="n">
+        <v>380.4</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>-1.092</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-1.392</v>
+      </c>
+      <c r="M5" t="n">
+        <v>9999.6</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-139.19</v>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -3521,7 +3680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5021,6 +5180,45 @@
         <v>3</v>
       </c>
       <c r="K38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>199432.79</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>199432.79</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-5.77</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-5.77</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>4</v>
+      </c>
+      <c r="K39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5035,7 +5233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6097,6 +6295,387 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7081EBE62C</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>607</v>
+      </c>
+      <c r="I23" t="n">
+        <v>16</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7081EBE62C</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>607</v>
+      </c>
+      <c r="I24" t="n">
+        <v>16</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AC11BADE6F</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>384.6</v>
+      </c>
+      <c r="I25" t="n">
+        <v>26</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AC11BADE6F</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>384.6</v>
+      </c>
+      <c r="I26" t="n">
+        <v>26</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>@ 2026-08-28 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>F7B517CE6D</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>374.98</v>
+      </c>
+      <c r="I27" t="n">
+        <v>26</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>4B505E99E9</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>389.21</v>
+      </c>
+      <c r="I28" t="n">
+        <v>13</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6742D7CAD5</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>395.37</v>
+      </c>
+      <c r="I29" t="n">
+        <v>13</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20:43:26</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0A87174464</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>26</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>time exit @ 380.40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-08-31T15:05 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2089,6 +2089,48 @@
       </c>
       <c r="L39" t="n">
         <v>37.7</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>500</v>
+      </c>
+      <c r="D40" t="n">
+        <v>500</v>
+      </c>
+      <c r="E40" t="n">
+        <v>500</v>
+      </c>
+      <c r="F40" t="n">
+        <v>8</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="n">
+        <v>8</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
+        <v>48.2</v>
       </c>
     </row>
   </sheetData>
@@ -2102,7 +2144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3306,6 +3348,486 @@
         <v>1</v>
       </c>
       <c r="P22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1260</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1249.92</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1218.67</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1264.92</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1284.92</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="M23" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="N23" t="n">
+        <v>1358.68</v>
+      </c>
+      <c r="O23" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1455.8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1444.15</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1408.05</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1461.48</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1484.59</v>
+      </c>
+      <c r="K24" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="M24" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1589.38</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AIIL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>551.6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>547.1900000000001</v>
+      </c>
+      <c r="H25" t="n">
+        <v>533.51</v>
+      </c>
+      <c r="I25" t="n">
+        <v>553.75</v>
+      </c>
+      <c r="J25" t="n">
+        <v>562.51</v>
+      </c>
+      <c r="K25" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="M25" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="N25" t="n">
+        <v>562.88</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>185.49</v>
+      </c>
+      <c r="G26" t="n">
+        <v>184.01</v>
+      </c>
+      <c r="H26" t="n">
+        <v>179.41</v>
+      </c>
+      <c r="I26" t="n">
+        <v>186.21</v>
+      </c>
+      <c r="J26" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="K26" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="M26" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="N26" t="n">
+        <v>202.96</v>
+      </c>
+      <c r="O26" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EIHOTEL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>282.1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>279.84</v>
+      </c>
+      <c r="H27" t="n">
+        <v>272.85</v>
+      </c>
+      <c r="I27" t="n">
+        <v>283.2</v>
+      </c>
+      <c r="J27" t="n">
+        <v>287.68</v>
+      </c>
+      <c r="K27" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="M27" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="N27" t="n">
+        <v>303.56</v>
+      </c>
+      <c r="O27" t="n">
+        <v>1</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>364</v>
+      </c>
+      <c r="G28" t="n">
+        <v>361.09</v>
+      </c>
+      <c r="H28" t="n">
+        <v>352.06</v>
+      </c>
+      <c r="I28" t="n">
+        <v>365.42</v>
+      </c>
+      <c r="J28" t="n">
+        <v>371.2</v>
+      </c>
+      <c r="K28" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="N28" t="n">
+        <v>399.32</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>710</v>
+      </c>
+      <c r="G29" t="n">
+        <v>704.3200000000001</v>
+      </c>
+      <c r="H29" t="n">
+        <v>686.71</v>
+      </c>
+      <c r="I29" t="n">
+        <v>712.77</v>
+      </c>
+      <c r="J29" t="n">
+        <v>724.04</v>
+      </c>
+      <c r="K29" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="M29" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="N29" t="n">
+        <v>726.61</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>HONAUT</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>35510</v>
+      </c>
+      <c r="G30" t="n">
+        <v>35225.92</v>
+      </c>
+      <c r="H30" t="n">
+        <v>34345.27</v>
+      </c>
+      <c r="I30" t="n">
+        <v>35648.63</v>
+      </c>
+      <c r="J30" t="n">
+        <v>36212.25</v>
+      </c>
+      <c r="K30" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M30" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="N30" t="n">
+        <v>37191.25</v>
+      </c>
+      <c r="O30" t="n">
+        <v>1</v>
+      </c>
+      <c r="P30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3680,7 +4202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5220,6 +5742,45 @@
       </c>
       <c r="K39" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>199432.79</v>
+      </c>
+      <c r="D40" t="n">
+        <v>8857.1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>190575.69</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-5.77</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-5.77</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>4</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5233,7 +5794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6676,6 +7237,246 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>4300E19DA9</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1265.3</v>
+      </c>
+      <c r="I31" t="n">
+        <v>7</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>4300E19DA9</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1265.3</v>
+      </c>
+      <c r="I32" t="n">
+        <v>7</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>@ 2026-08-31 11:30:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>120C1A7E62</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>1233.66</v>
+      </c>
+      <c r="I33" t="n">
+        <v>7</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>E05FC0E822</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1280.48</v>
+      </c>
+      <c r="I34" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:05:27</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CE729F36A4</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1300.72</v>
+      </c>
+      <c r="I35" t="n">
+        <v>4</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-08-31T22:46 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2131,6 +2131,48 @@
       </c>
       <c r="L40" t="n">
         <v>48.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>500</v>
+      </c>
+      <c r="D41" t="n">
+        <v>500</v>
+      </c>
+      <c r="E41" t="n">
+        <v>500</v>
+      </c>
+      <c r="F41" t="n">
+        <v>12</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>12</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -2144,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3828,6 +3870,726 @@
         <v>1</v>
       </c>
       <c r="P30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>33320</v>
+      </c>
+      <c r="G31" t="n">
+        <v>33053.44</v>
+      </c>
+      <c r="H31" t="n">
+        <v>32227.1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>33450.08</v>
+      </c>
+      <c r="J31" t="n">
+        <v>33978.94</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="M31" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="N31" t="n">
+        <v>34912</v>
+      </c>
+      <c r="O31" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>198</v>
+      </c>
+      <c r="G32" t="n">
+        <v>196.42</v>
+      </c>
+      <c r="H32" t="n">
+        <v>191.51</v>
+      </c>
+      <c r="I32" t="n">
+        <v>198.77</v>
+      </c>
+      <c r="J32" t="n">
+        <v>201.92</v>
+      </c>
+      <c r="K32" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="N32" t="n">
+        <v>206.98</v>
+      </c>
+      <c r="O32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2859.1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2836.23</v>
+      </c>
+      <c r="H33" t="n">
+        <v>2765.32</v>
+      </c>
+      <c r="I33" t="n">
+        <v>2870.26</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2915.64</v>
+      </c>
+      <c r="K33" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="N33" t="n">
+        <v>3027.32</v>
+      </c>
+      <c r="O33" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1214.9</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1205.18</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1175.05</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1219.64</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1238.93</v>
+      </c>
+      <c r="K34" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1329.41</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1593.1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1580.36</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1540.85</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1599.32</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1624.61</v>
+      </c>
+      <c r="K35" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1684.98</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1811.9</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1797.4</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1752.47</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1818.97</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1847.73</v>
+      </c>
+      <c r="K36" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1933.01</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1079.8</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1071.16</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1044.38</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1084.02</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1101.15</v>
+      </c>
+      <c r="K37" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M37" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="N37" t="n">
+        <v>1119.09</v>
+      </c>
+      <c r="O37" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GMRAIRPORT</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>93.63</v>
+      </c>
+      <c r="G38" t="n">
+        <v>92.88</v>
+      </c>
+      <c r="H38" t="n">
+        <v>90.56</v>
+      </c>
+      <c r="I38" t="n">
+        <v>94</v>
+      </c>
+      <c r="J38" t="n">
+        <v>95.48</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="N38" t="n">
+        <v>102.06</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>255.5</v>
+      </c>
+      <c r="G39" t="n">
+        <v>253.46</v>
+      </c>
+      <c r="H39" t="n">
+        <v>247.12</v>
+      </c>
+      <c r="I39" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>260.55</v>
+      </c>
+      <c r="K39" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="N39" t="n">
+        <v>274.77</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>LATENTVIEW</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>269.8</v>
+      </c>
+      <c r="G40" t="n">
+        <v>267.64</v>
+      </c>
+      <c r="H40" t="n">
+        <v>260.95</v>
+      </c>
+      <c r="I40" t="n">
+        <v>270.85</v>
+      </c>
+      <c r="J40" t="n">
+        <v>275.14</v>
+      </c>
+      <c r="K40" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="M40" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N40" t="n">
+        <v>285.04</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>VTL</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>572.05</v>
+      </c>
+      <c r="G41" t="n">
+        <v>567.47</v>
+      </c>
+      <c r="H41" t="n">
+        <v>553.29</v>
+      </c>
+      <c r="I41" t="n">
+        <v>574.28</v>
+      </c>
+      <c r="J41" t="n">
+        <v>583.36</v>
+      </c>
+      <c r="K41" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M41" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="N41" t="n">
+        <v>592.48</v>
+      </c>
+      <c r="O41" t="n">
+        <v>1</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ZENSARTECH</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>460.35</v>
+      </c>
+      <c r="G42" t="n">
+        <v>456.67</v>
+      </c>
+      <c r="H42" t="n">
+        <v>445.25</v>
+      </c>
+      <c r="I42" t="n">
+        <v>462.15</v>
+      </c>
+      <c r="J42" t="n">
+        <v>469.45</v>
+      </c>
+      <c r="K42" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="M42" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="N42" t="n">
+        <v>486.64</v>
+      </c>
+      <c r="O42" t="n">
+        <v>1</v>
+      </c>
+      <c r="P42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3842,7 +4604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4145,6 +4907,63 @@
         <v>-139.19</v>
       </c>
       <c r="O5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1265.3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1233.66</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1280.48</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1300.72</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1260</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.419</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-0.719</v>
+      </c>
+      <c r="M6" t="n">
+        <v>8857.1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-63.68</v>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -4202,7 +5021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5781,6 +6600,45 @@
       </c>
       <c r="K40" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>199369.11</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>199369.11</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-6.49</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-6.49</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>5</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5794,7 +6652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7477,6 +8335,51 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>22:45:43</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>6126438D35</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>7</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>time exit @ 1260.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-01T14:01 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2173,6 +2173,48 @@
       </c>
       <c r="L41" t="n">
         <v>42</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>500</v>
+      </c>
+      <c r="D42" t="n">
+        <v>500</v>
+      </c>
+      <c r="E42" t="n">
+        <v>500</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" t="n">
+        <v>5</v>
+      </c>
+      <c r="I42" t="n">
+        <v>4</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>28.4</v>
       </c>
     </row>
   </sheetData>
@@ -2186,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4590,6 +4632,306 @@
         <v>1</v>
       </c>
       <c r="P42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1379.7</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1368.66</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1334.45</v>
+      </c>
+      <c r="I43" t="n">
+        <v>1385.09</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1406.98</v>
+      </c>
+      <c r="K43" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M43" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="N43" t="n">
+        <v>1574.14</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1</v>
+      </c>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>595.75</v>
+      </c>
+      <c r="G44" t="n">
+        <v>590.98</v>
+      </c>
+      <c r="H44" t="n">
+        <v>576.21</v>
+      </c>
+      <c r="I44" t="n">
+        <v>598.08</v>
+      </c>
+      <c r="J44" t="n">
+        <v>607.53</v>
+      </c>
+      <c r="K44" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M44" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="N44" t="n">
+        <v>615.72</v>
+      </c>
+      <c r="O44" t="n">
+        <v>1</v>
+      </c>
+      <c r="P44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>GABRIEL</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1412.8</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1401.5</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1366.46</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1418.32</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1440.74</v>
+      </c>
+      <c r="K45" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="M45" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="N45" t="n">
+        <v>1443.87</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>280.3</v>
+      </c>
+      <c r="G46" t="n">
+        <v>278.06</v>
+      </c>
+      <c r="H46" t="n">
+        <v>271.11</v>
+      </c>
+      <c r="I46" t="n">
+        <v>281.39</v>
+      </c>
+      <c r="J46" t="n">
+        <v>285.84</v>
+      </c>
+      <c r="K46" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="M46" t="n">
+        <v>35</v>
+      </c>
+      <c r="N46" t="n">
+        <v>296.43</v>
+      </c>
+      <c r="O46" t="n">
+        <v>1</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>12942</v>
+      </c>
+      <c r="G47" t="n">
+        <v>12838.46</v>
+      </c>
+      <c r="H47" t="n">
+        <v>12517.5</v>
+      </c>
+      <c r="I47" t="n">
+        <v>12992.53</v>
+      </c>
+      <c r="J47" t="n">
+        <v>13197.94</v>
+      </c>
+      <c r="K47" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="M47" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="N47" t="n">
+        <v>13718.25</v>
+      </c>
+      <c r="O47" t="n">
+        <v>1</v>
+      </c>
+      <c r="P47" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4604,7 +4946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4964,6 +5306,120 @@
         <v>-63.68</v>
       </c>
       <c r="O6" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1444.15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1408.05</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1461.48</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1484.59</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1408.05</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="M7" t="n">
+        <v>8664.9</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-242.62</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>184.01</v>
+      </c>
+      <c r="E8" t="n">
+        <v>54</v>
+      </c>
+      <c r="F8" t="n">
+        <v>179.41</v>
+      </c>
+      <c r="G8" t="n">
+        <v>186.21</v>
+      </c>
+      <c r="H8" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="I8" t="n">
+        <v>179.41</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="M8" t="n">
+        <v>9936.540000000001</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-278.22</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -5021,7 +5477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6639,6 +7095,45 @@
       </c>
       <c r="K41" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:01:30</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>198848.27</v>
+      </c>
+      <c r="D42" t="n">
+        <v>42913.92</v>
+      </c>
+      <c r="E42" t="n">
+        <v>155934.35</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-12.09</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-12.09</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>7</v>
+      </c>
+      <c r="K42" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -6652,7 +7147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8380,6 +8875,2166 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5E5F919BCC</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1444.15</v>
+      </c>
+      <c r="I37" t="n">
+        <v>6</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5E5F919BCC</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1444.15</v>
+      </c>
+      <c r="I38" t="n">
+        <v>6</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>@ 2026-09-01 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>8EBFD21429</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>1408.05</v>
+      </c>
+      <c r="I39" t="n">
+        <v>6</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>3D7A0BD8B6</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1461.48</v>
+      </c>
+      <c r="I40" t="n">
+        <v>3</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7FDE8C2DE3</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1484.59</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:01:25</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>57AAF6BBB0</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>1408.05</v>
+      </c>
+      <c r="I42" t="n">
+        <v>6</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>STOP_LOSS close 1403.80 low 1401.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>C23EB405AB</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>AIIL</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>547.1900000000001</v>
+      </c>
+      <c r="I43" t="n">
+        <v>18</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>gap-up open 568.90 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>DA773C9D04</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>184.01</v>
+      </c>
+      <c r="I44" t="n">
+        <v>54</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DA773C9D04</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>184.01</v>
+      </c>
+      <c r="I45" t="n">
+        <v>54</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>@ 2026-09-01 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>392A113D48</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>179.41</v>
+      </c>
+      <c r="I46" t="n">
+        <v>54</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>E20B153FD4</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>186.21</v>
+      </c>
+      <c r="I47" t="n">
+        <v>27</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>A87F4576C8</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="I48" t="n">
+        <v>27</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>8D6315D322</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FIRSTCRY</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>179.41</v>
+      </c>
+      <c r="I49" t="n">
+        <v>54</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>STOP_LOSS close 178.47 low 177.46</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2B060B938E</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>EIHOTEL</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>279.84</v>
+      </c>
+      <c r="I50" t="n">
+        <v>35</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>14:01:26</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2B060B938E</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>EIHOTEL</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>279.84</v>
+      </c>
+      <c r="I51" t="n">
+        <v>35</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>A383A5E303</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>361.09</v>
+      </c>
+      <c r="I52" t="n">
+        <v>27</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>A383A5E303</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>EMAMILTD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>361.09</v>
+      </c>
+      <c r="I53" t="n">
+        <v>27</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>86C4B8988E</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>704.3200000000001</v>
+      </c>
+      <c r="I54" t="n">
+        <v>14</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>86C4B8988E</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>704.3200000000001</v>
+      </c>
+      <c r="I55" t="n">
+        <v>14</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>@ 2026-09-01 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>123809D95D</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>686.71</v>
+      </c>
+      <c r="I56" t="n">
+        <v>14</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>8ED7E6C9F8</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>712.77</v>
+      </c>
+      <c r="I57" t="n">
+        <v>7</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>035952FE4C</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>724.04</v>
+      </c>
+      <c r="I58" t="n">
+        <v>7</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>9959E7A736</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>712.77</v>
+      </c>
+      <c r="I59" t="n">
+        <v>7</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>T1 50% booked</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>14:01:27</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>53F0E38AAD</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>704.3200000000001</v>
+      </c>
+      <c r="I60" t="n">
+        <v>7</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>SL shifted to breakeven</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>03FCB91AEC</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>HONAUT</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>35225.92</v>
+      </c>
+      <c r="I61" t="n">
+        <v>1</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>03FCB91AEC</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>HONAUT</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>35225.92</v>
+      </c>
+      <c r="I62" t="n">
+        <v>1</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>B7C4112AB3</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>33053.44</v>
+      </c>
+      <c r="I63" t="n">
+        <v>1</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>B7C4112AB3</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>33053.44</v>
+      </c>
+      <c r="I64" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>@ 2026-09-01 13:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>8A86559CFF</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>32227.1</v>
+      </c>
+      <c r="I65" t="n">
+        <v>1</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>997DA39203</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>33450.08</v>
+      </c>
+      <c r="I66" t="n">
+        <v>1</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>472DF2C18B</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>33978.94</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>14:01:28</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>EAB57B2EC8</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>196.42</v>
+      </c>
+      <c r="I68" t="n">
+        <v>50</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>gap-up open 203.06 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>69ADA6C184</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>2836.23</v>
+      </c>
+      <c r="I69" t="n">
+        <v>3</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>gap-up open 2915.00 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>3ECD167532</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1205.18</v>
+      </c>
+      <c r="I70" t="n">
+        <v>8</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>gap-up open 1226.20 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>8D4A3556D3</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>1580.36</v>
+      </c>
+      <c r="I71" t="n">
+        <v>6</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>gap-up open 1633.20 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>23F63CC65A</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>1797.4</v>
+      </c>
+      <c r="I72" t="n">
+        <v>5</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>gap-up open 1852.90 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>6490C40354</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>1071.16</v>
+      </c>
+      <c r="I73" t="n">
+        <v>9</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>gap-up open 1088.70 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>0763EACD70</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>GMRAIRPORT</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>92.88</v>
+      </c>
+      <c r="I74" t="n">
+        <v>107</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>gap-up open 95.75 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>5262FAD389</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>253.46</v>
+      </c>
+      <c r="I75" t="n">
+        <v>39</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>gap-up open 261.50 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>14:01:29</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>B1CC86B769</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>LATENTVIEW</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>267.64</v>
+      </c>
+      <c r="I76" t="n">
+        <v>37</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>14:01:30</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>B1CC86B769</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>LATENTVIEW</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>267.64</v>
+      </c>
+      <c r="I77" t="n">
+        <v>37</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>14:01:30</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>8462C4D6E0</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>VTL</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>567.47</v>
+      </c>
+      <c r="I78" t="n">
+        <v>17</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>14:01:30</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>8462C4D6E0</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>VTL</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>567.47</v>
+      </c>
+      <c r="I79" t="n">
+        <v>17</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>14:01:30</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>F90CB0145B</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ZENSARTECH</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>456.67</v>
+      </c>
+      <c r="I80" t="n">
+        <v>21</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>14:01:30</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>F90CB0145B</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>ZENSARTECH</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>456.67</v>
+      </c>
+      <c r="I81" t="n">
+        <v>21</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-01T19:14 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2215,6 +2215,48 @@
       </c>
       <c r="L42" t="n">
         <v>28.4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>500</v>
+      </c>
+      <c r="D43" t="n">
+        <v>500</v>
+      </c>
+      <c r="E43" t="n">
+        <v>500</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>54.9</v>
       </c>
     </row>
   </sheetData>
@@ -2228,7 +2270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4932,6 +4974,186 @@
         <v>1</v>
       </c>
       <c r="P47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>242.36</v>
+      </c>
+      <c r="G48" t="n">
+        <v>240.42</v>
+      </c>
+      <c r="H48" t="n">
+        <v>234.41</v>
+      </c>
+      <c r="I48" t="n">
+        <v>243.31</v>
+      </c>
+      <c r="J48" t="n">
+        <v>247.15</v>
+      </c>
+      <c r="K48" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="M48" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="N48" t="n">
+        <v>251.87</v>
+      </c>
+      <c r="O48" t="n">
+        <v>1</v>
+      </c>
+      <c r="P48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>5348</v>
+      </c>
+      <c r="G49" t="n">
+        <v>5305.22</v>
+      </c>
+      <c r="H49" t="n">
+        <v>5172.59</v>
+      </c>
+      <c r="I49" t="n">
+        <v>5368.88</v>
+      </c>
+      <c r="J49" t="n">
+        <v>5453.76</v>
+      </c>
+      <c r="K49" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="M49" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="N49" t="n">
+        <v>5634.14</v>
+      </c>
+      <c r="O49" t="n">
+        <v>1</v>
+      </c>
+      <c r="P49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>8895.5</v>
+      </c>
+      <c r="G50" t="n">
+        <v>8824.34</v>
+      </c>
+      <c r="H50" t="n">
+        <v>8603.73</v>
+      </c>
+      <c r="I50" t="n">
+        <v>8930.23</v>
+      </c>
+      <c r="J50" t="n">
+        <v>9071.42</v>
+      </c>
+      <c r="K50" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="M50" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="N50" t="n">
+        <v>9170.92</v>
+      </c>
+      <c r="O50" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4946,7 +5168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5420,6 +5642,120 @@
         <v>-278.22</v>
       </c>
       <c r="O8" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>704.3200000000001</v>
+      </c>
+      <c r="E9" t="n">
+        <v>14</v>
+      </c>
+      <c r="F9" t="n">
+        <v>686.71</v>
+      </c>
+      <c r="G9" t="n">
+        <v>712.77</v>
+      </c>
+      <c r="H9" t="n">
+        <v>724.04</v>
+      </c>
+      <c r="I9" t="n">
+        <v>711.9</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1.138</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="M9" t="n">
+        <v>9860.48</v>
+      </c>
+      <c r="N9" t="n">
+        <v>82.63</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>33053.44</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>32227.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>33450.08</v>
+      </c>
+      <c r="H10" t="n">
+        <v>33978.94</v>
+      </c>
+      <c r="I10" t="n">
+        <v>33315</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="M10" t="n">
+        <v>33053.44</v>
+      </c>
+      <c r="N10" t="n">
+        <v>162.29</v>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -5477,7 +5813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7134,6 +7470,45 @@
       </c>
       <c r="K42" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>199093.19</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>199093.19</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="I43" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J43" t="n">
+        <v>9</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7147,7 +7522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11035,6 +11410,96 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>A5276AE588</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>14</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>time exit @ 711.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>19:13:46</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>6BCD32E0DA</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>3MINDIA</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>1</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>time exit @ 33315.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-02T13:19 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2257,6 +2257,48 @@
       </c>
       <c r="L43" t="n">
         <v>54.9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>13:18:47</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>500</v>
+      </c>
+      <c r="D44" t="n">
+        <v>500</v>
+      </c>
+      <c r="E44" t="n">
+        <v>500</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" t="n">
+        <v>7</v>
+      </c>
+      <c r="H44" t="n">
+        <v>3</v>
+      </c>
+      <c r="I44" t="n">
+        <v>7</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>28.7</v>
       </c>
     </row>
   </sheetData>
@@ -2270,7 +2312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P50"/>
+  <dimension ref="A1:P53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5154,6 +5196,186 @@
         <v>1</v>
       </c>
       <c r="P50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>13:18:47</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>7573.5</v>
+      </c>
+      <c r="G51" t="n">
+        <v>7512.91</v>
+      </c>
+      <c r="H51" t="n">
+        <v>7325.09</v>
+      </c>
+      <c r="I51" t="n">
+        <v>7603.07</v>
+      </c>
+      <c r="J51" t="n">
+        <v>7723.27</v>
+      </c>
+      <c r="K51" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="M51" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="N51" t="n">
+        <v>8004.1</v>
+      </c>
+      <c r="O51" t="n">
+        <v>1</v>
+      </c>
+      <c r="P51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>13:18:47</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>5232.5</v>
+      </c>
+      <c r="G52" t="n">
+        <v>5190.64</v>
+      </c>
+      <c r="H52" t="n">
+        <v>5060.87</v>
+      </c>
+      <c r="I52" t="n">
+        <v>5252.93</v>
+      </c>
+      <c r="J52" t="n">
+        <v>5335.98</v>
+      </c>
+      <c r="K52" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.206</v>
+      </c>
+      <c r="M52" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="N52" t="n">
+        <v>5675.18</v>
+      </c>
+      <c r="O52" t="n">
+        <v>1</v>
+      </c>
+      <c r="P52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>13:18:47</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>2662.3</v>
+      </c>
+      <c r="G53" t="n">
+        <v>2641</v>
+      </c>
+      <c r="H53" t="n">
+        <v>2574.98</v>
+      </c>
+      <c r="I53" t="n">
+        <v>2672.69</v>
+      </c>
+      <c r="J53" t="n">
+        <v>2714.95</v>
+      </c>
+      <c r="K53" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="M53" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="N53" t="n">
+        <v>2821.32</v>
+      </c>
+      <c r="O53" t="n">
+        <v>1</v>
+      </c>
+      <c r="P53" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5813,7 +6035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7509,6 +7731,45 @@
       </c>
       <c r="K43" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>13:18:53</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>199093.19</v>
+      </c>
+      <c r="D44" t="n">
+        <v>65593.64</v>
+      </c>
+      <c r="E44" t="n">
+        <v>133499.55</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="I44" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J44" t="n">
+        <v>9</v>
+      </c>
+      <c r="K44" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -7522,7 +7783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11500,6 +11761,1830 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>13:18:47</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>B0B0C8997E</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>1368.66</v>
+      </c>
+      <c r="I84" t="n">
+        <v>7</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>13:18:47</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>B0B0C8997E</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>1368.66</v>
+      </c>
+      <c r="I85" t="n">
+        <v>7</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>7EE8EC959D</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>1334.45</v>
+      </c>
+      <c r="I86" t="n">
+        <v>7</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>EDB1A22D8C</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>1385.09</v>
+      </c>
+      <c r="I87" t="n">
+        <v>3</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>796D73BFBB</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>1406.98</v>
+      </c>
+      <c r="I88" t="n">
+        <v>4</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>7A1758C776</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>1385.09</v>
+      </c>
+      <c r="I89" t="n">
+        <v>3</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>T1 50% booked</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>EC29FF0684</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>1368.66</v>
+      </c>
+      <c r="I90" t="n">
+        <v>4</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>SL shifted to breakeven</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2582412751</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>590.98</v>
+      </c>
+      <c r="I91" t="n">
+        <v>16</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>13:18:48</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2582412751</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>590.98</v>
+      </c>
+      <c r="I92" t="n">
+        <v>16</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 10:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>13:18:49</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2165984081</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>576.21</v>
+      </c>
+      <c r="I93" t="n">
+        <v>16</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>13:18:49</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>EAEF9E385F</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>598.08</v>
+      </c>
+      <c r="I94" t="n">
+        <v>8</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>13:18:49</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>DD06E10633</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>607.53</v>
+      </c>
+      <c r="I95" t="n">
+        <v>8</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>13:18:49</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>858337B2BF</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>GABRIEL</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>1401.5</v>
+      </c>
+      <c r="I96" t="n">
+        <v>7</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>gap-up open 1425.00 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>13:18:49</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>18B12C99CB</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>278.06</v>
+      </c>
+      <c r="I97" t="n">
+        <v>35</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13:18:49</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>18B12C99CB</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>278.06</v>
+      </c>
+      <c r="I98" t="n">
+        <v>35</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>95188FDF2F</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
+        <v>271.11</v>
+      </c>
+      <c r="I99" t="n">
+        <v>35</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>BB0550A143</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>281.39</v>
+      </c>
+      <c r="I100" t="n">
+        <v>17</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>810CA0AA80</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>285.84</v>
+      </c>
+      <c r="I101" t="n">
+        <v>18</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>5553316DAF</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>12838.46</v>
+      </c>
+      <c r="I102" t="n">
+        <v>1</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>5553316DAF</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>12838.46</v>
+      </c>
+      <c r="I103" t="n">
+        <v>1</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>67FCFBBD5D</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H104" t="n">
+        <v>12517.5</v>
+      </c>
+      <c r="I104" t="n">
+        <v>1</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>13:18:50</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>E1B5099761</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>12992.53</v>
+      </c>
+      <c r="I105" t="n">
+        <v>1</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>13:18:51</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>D3E3161E66</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>13197.94</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>13:18:51</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>4A44627128</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>240.42</v>
+      </c>
+      <c r="I107" t="n">
+        <v>41</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>13:18:51</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>4A44627128</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>240.42</v>
+      </c>
+      <c r="I108" t="n">
+        <v>41</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>13:18:51</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>6E9978523B</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>234.41</v>
+      </c>
+      <c r="I109" t="n">
+        <v>41</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>13:18:51</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>1781D005CF</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>243.31</v>
+      </c>
+      <c r="I110" t="n">
+        <v>20</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>13:18:51</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>C2591AA017</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>247.15</v>
+      </c>
+      <c r="I111" t="n">
+        <v>21</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>13:18:52</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>EBBBB224FA</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>5305.22</v>
+      </c>
+      <c r="I112" t="n">
+        <v>1</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>13:18:52</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>EBBBB224FA</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>5305.22</v>
+      </c>
+      <c r="I113" t="n">
+        <v>1</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>13:18:52</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>3684A8B38D</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H114" t="n">
+        <v>5172.59</v>
+      </c>
+      <c r="I114" t="n">
+        <v>1</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>13:18:52</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>1F5EF26E5D</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>5368.88</v>
+      </c>
+      <c r="I115" t="n">
+        <v>1</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>13:18:52</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>A6C040C4D1</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>5453.76</v>
+      </c>
+      <c r="I116" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>13:18:52</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>699B1C88D6</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>8824.34</v>
+      </c>
+      <c r="I117" t="n">
+        <v>1</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>13:18:53</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>699B1C88D6</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>8824.34</v>
+      </c>
+      <c r="I118" t="n">
+        <v>1</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>@ 2026-09-02 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>13:18:53</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>D9F7E98A27</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>8603.73</v>
+      </c>
+      <c r="I119" t="n">
+        <v>1</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>13:18:53</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>C1729F3EFA</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>8930.23</v>
+      </c>
+      <c r="I120" t="n">
+        <v>1</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>13:18:53</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>88C7967919</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>9071.42</v>
+      </c>
+      <c r="I121" t="n">
+        <v>0</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-02T18:12 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2299,6 +2299,48 @@
       </c>
       <c r="L44" t="n">
         <v>28.7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>18:12:34</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>500</v>
+      </c>
+      <c r="D45" t="n">
+        <v>500</v>
+      </c>
+      <c r="E45" t="n">
+        <v>500</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>7</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2312,7 +2354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5376,6 +5418,186 @@
         <v>1</v>
       </c>
       <c r="P53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>18:12:34</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AIIL</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>507.45</v>
+      </c>
+      <c r="G54" t="n">
+        <v>503.39</v>
+      </c>
+      <c r="H54" t="n">
+        <v>490.81</v>
+      </c>
+      <c r="I54" t="n">
+        <v>509.43</v>
+      </c>
+      <c r="J54" t="n">
+        <v>517.49</v>
+      </c>
+      <c r="K54" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="M54" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N54" t="n">
+        <v>559.08</v>
+      </c>
+      <c r="O54" t="n">
+        <v>1</v>
+      </c>
+      <c r="P54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>18:12:34</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G55" t="n">
+        <v>5128.64</v>
+      </c>
+      <c r="H55" t="n">
+        <v>5000.42</v>
+      </c>
+      <c r="I55" t="n">
+        <v>5190.18</v>
+      </c>
+      <c r="J55" t="n">
+        <v>5272.24</v>
+      </c>
+      <c r="K55" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="M55" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="N55" t="n">
+        <v>5613.79</v>
+      </c>
+      <c r="O55" t="n">
+        <v>1</v>
+      </c>
+      <c r="P55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>18:12:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>VOLTAS</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1152.1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1142.88</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1114.31</v>
+      </c>
+      <c r="I56" t="n">
+        <v>1156.6</v>
+      </c>
+      <c r="J56" t="n">
+        <v>1174.88</v>
+      </c>
+      <c r="K56" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="M56" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="N56" t="n">
+        <v>1243.82</v>
+      </c>
+      <c r="O56" t="n">
+        <v>1</v>
+      </c>
+      <c r="P56" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5390,7 +5612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5978,6 +6200,405 @@
         <v>162.29</v>
       </c>
       <c r="O10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1368.66</v>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1334.45</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1385.09</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1406.98</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1396.6</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1.621</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1.321</v>
+      </c>
+      <c r="M11" t="n">
+        <v>9580.620000000001</v>
+      </c>
+      <c r="N11" t="n">
+        <v>126.56</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>590.98</v>
+      </c>
+      <c r="E12" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" t="n">
+        <v>576.21</v>
+      </c>
+      <c r="G12" t="n">
+        <v>598.08</v>
+      </c>
+      <c r="H12" t="n">
+        <v>607.53</v>
+      </c>
+      <c r="I12" t="n">
+        <v>589</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>-0.335</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-0.635</v>
+      </c>
+      <c r="M12" t="n">
+        <v>9455.68</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-60.04</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>278.06</v>
+      </c>
+      <c r="E13" t="n">
+        <v>35</v>
+      </c>
+      <c r="F13" t="n">
+        <v>271.11</v>
+      </c>
+      <c r="G13" t="n">
+        <v>281.39</v>
+      </c>
+      <c r="H13" t="n">
+        <v>285.84</v>
+      </c>
+      <c r="I13" t="n">
+        <v>282.15</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1.334</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="M13" t="n">
+        <v>9732.1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>100.63</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>12838.46</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12517.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>12992.53</v>
+      </c>
+      <c r="H14" t="n">
+        <v>13197.94</v>
+      </c>
+      <c r="I14" t="n">
+        <v>12849</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-0.218</v>
+      </c>
+      <c r="M14" t="n">
+        <v>12838.46</v>
+      </c>
+      <c r="N14" t="n">
+        <v>-27.99</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>240.42</v>
+      </c>
+      <c r="E15" t="n">
+        <v>41</v>
+      </c>
+      <c r="F15" t="n">
+        <v>234.41</v>
+      </c>
+      <c r="G15" t="n">
+        <v>243.31</v>
+      </c>
+      <c r="H15" t="n">
+        <v>247.15</v>
+      </c>
+      <c r="I15" t="n">
+        <v>239.37</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>-0.437</v>
+      </c>
+      <c r="L15" t="n">
+        <v>-0.737</v>
+      </c>
+      <c r="M15" t="n">
+        <v>9857.219999999999</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-72.65000000000001</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5305.22</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>5172.59</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5368.88</v>
+      </c>
+      <c r="H16" t="n">
+        <v>5453.76</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5172.59</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="M16" t="n">
+        <v>5305.22</v>
+      </c>
+      <c r="N16" t="n">
+        <v>-148.55</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>8824.34</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8603.73</v>
+      </c>
+      <c r="G17" t="n">
+        <v>8930.23</v>
+      </c>
+      <c r="H17" t="n">
+        <v>9071.42</v>
+      </c>
+      <c r="I17" t="n">
+        <v>8804</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="M17" t="n">
+        <v>8824.34</v>
+      </c>
+      <c r="N17" t="n">
+        <v>-46.77</v>
+      </c>
+      <c r="O17" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -6035,7 +6656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7770,6 +8391,45 @@
       </c>
       <c r="K44" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>18:12:36</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>198964.38</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>198964.38</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-13.32</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-13.32</v>
+      </c>
+      <c r="I45" t="n">
+        <v>25</v>
+      </c>
+      <c r="J45" t="n">
+        <v>16</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7783,7 +8443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13585,6 +14245,420 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>BDC35954E3</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>7</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>time exit @ 1396.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>2F9E4413FD</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>BIKAJI</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>16</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>time exit @ 589.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>C105EAB3C7</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>281.39</v>
+      </c>
+      <c r="I124" t="n">
+        <v>17</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>T1 50% booked</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>3CB03D75E6</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H125" t="n">
+        <v>278.06</v>
+      </c>
+      <c r="I125" t="n">
+        <v>18</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>SL shifted to breakeven</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>E903CCA886</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>JAINREC</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>35</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>time exit @ 282.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>412094F6F6</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>1</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>time exit @ 12849.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>18:12:35</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>6B3A2607BC</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>JWL</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>41</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>time exit @ 239.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>18:12:36</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>923504D9C3</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H129" t="n">
+        <v>5172.59</v>
+      </c>
+      <c r="I129" t="n">
+        <v>1</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>STOP_LOSS close 5165.00 low 5164.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>18:12:36</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>A07C8C8638</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>1</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>time exit @ 8804.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-03T13:27 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2341,6 +2341,48 @@
       </c>
       <c r="L45" t="n">
         <v>31</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>13:27:24</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>500</v>
+      </c>
+      <c r="D46" t="n">
+        <v>500</v>
+      </c>
+      <c r="E46" t="n">
+        <v>500</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>28.2</v>
       </c>
     </row>
   </sheetData>
@@ -2354,7 +2396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P56"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5598,6 +5640,66 @@
         <v>1</v>
       </c>
       <c r="P56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>13:27:24</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>DEEPAKFERT</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1366.3</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1355.37</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1321.49</v>
+      </c>
+      <c r="I57" t="n">
+        <v>1371.63</v>
+      </c>
+      <c r="J57" t="n">
+        <v>1393.32</v>
+      </c>
+      <c r="K57" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="M57" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="N57" t="n">
+        <v>1463.73</v>
+      </c>
+      <c r="O57" t="n">
+        <v>1</v>
+      </c>
+      <c r="P57" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6656,7 +6758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8430,6 +8532,45 @@
       </c>
       <c r="K45" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>13:27:26</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>198964.38</v>
+      </c>
+      <c r="D46" t="n">
+        <v>7923</v>
+      </c>
+      <c r="E46" t="n">
+        <v>191041.38</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-13.32</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-13.32</v>
+      </c>
+      <c r="I46" t="n">
+        <v>25</v>
+      </c>
+      <c r="J46" t="n">
+        <v>16</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -8443,7 +8584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K130"/>
+  <dimension ref="A1:K141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14659,6 +14800,534 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:27:24</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>1A3146B0F0</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>7512.91</v>
+      </c>
+      <c r="I131" t="n">
+        <v>1</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>gap-up open 7730.00 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>13:27:25</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>2BE077FE86</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>5190.64</v>
+      </c>
+      <c r="I132" t="n">
+        <v>1</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>gap-up open 5305.00 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>13:27:25</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>E29D82D20B</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>2641</v>
+      </c>
+      <c r="I133" t="n">
+        <v>3</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:27:25</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>E29D82D20B</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>2641</v>
+      </c>
+      <c r="I134" t="n">
+        <v>3</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>@ 2026-09-03 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:27:25</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>87AB8338F9</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>SL-M</t>
+        </is>
+      </c>
+      <c r="H135" t="n">
+        <v>2574.98</v>
+      </c>
+      <c r="I135" t="n">
+        <v>3</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>protective SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:27:25</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>9343FDE8A8</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>2672.69</v>
+      </c>
+      <c r="I136" t="n">
+        <v>1</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>T1 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:27:25</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>B077402123</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>2714.95</v>
+      </c>
+      <c r="I137" t="n">
+        <v>2</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>T2 rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>13:27:26</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>6613DC2270</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>AIIL</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>503.39</v>
+      </c>
+      <c r="I138" t="n">
+        <v>19</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>gap-up open 515.00 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:27:26</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>C05103847F</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>KEI</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
+        <v>5128.64</v>
+      </c>
+      <c r="I139" t="n">
+        <v>1</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>gap-up open 5223.50 &gt; entry*1.015</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:27:26</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>179069A6FE</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>VOLTAS</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
+        <v>1142.88</v>
+      </c>
+      <c r="I140" t="n">
+        <v>8</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ENTRY MIS DAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>13:27:26</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>179069A6FE</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>VOLTAS</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>1142.88</v>
+      </c>
+      <c r="I141" t="n">
+        <v>8</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>CANCELLED</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>DAY expired unfilled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-03T18:17 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2383,6 +2383,48 @@
       </c>
       <c r="L46" t="n">
         <v>28.2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>18:17:34</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>500</v>
+      </c>
+      <c r="D47" t="n">
+        <v>500</v>
+      </c>
+      <c r="E47" t="n">
+        <v>500</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>52.5</v>
       </c>
     </row>
   </sheetData>
@@ -2396,7 +2438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5700,6 +5742,126 @@
         <v>1</v>
       </c>
       <c r="P57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>18:17:35</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>OLECTRA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1244.8</v>
+      </c>
+      <c r="G58" t="n">
+        <v>1234.84</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1203.97</v>
+      </c>
+      <c r="I58" t="n">
+        <v>1249.66</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1269.42</v>
+      </c>
+      <c r="K58" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="M58" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="N58" t="n">
+        <v>1318.02</v>
+      </c>
+      <c r="O58" t="n">
+        <v>1</v>
+      </c>
+      <c r="P58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>18:17:35</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>UBL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1284.2</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1273.93</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1242.08</v>
+      </c>
+      <c r="I59" t="n">
+        <v>1289.21</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1309.6</v>
+      </c>
+      <c r="K59" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="M59" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="N59" t="n">
+        <v>1350.86</v>
+      </c>
+      <c r="O59" t="n">
+        <v>1</v>
+      </c>
+      <c r="P59" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5714,7 +5876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6701,6 +6863,63 @@
         <v>-46.77</v>
       </c>
       <c r="O17" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2641</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2574.98</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2672.69</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2714.95</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2630</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>TIME_EXIT</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>-0.417</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-0.717</v>
+      </c>
+      <c r="M18" t="n">
+        <v>7923</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-56.81</v>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -6758,7 +6977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8571,6 +8790,45 @@
       </c>
       <c r="K46" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>18:17:35</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>198907.57</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>198907.57</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-14.04</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-14.04</v>
+      </c>
+      <c r="I47" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J47" t="n">
+        <v>17</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8584,7 +8842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K141"/>
+  <dimension ref="A1:K142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15328,6 +15586,51 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>18:17:35</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>5177782FFB</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>RRKABEL</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>3</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>time exit @ 2630.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-04T10:49 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -432,111 +432,111 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U105"/>
+  <dimension ref="A1:U121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Stocks_Scanned</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Daily_Ok</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Intraday_Ok</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Signals_Found</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Tradeable</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Watchlist</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Errors</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Duration_Sec</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Upper_Band</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Qualifies</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Rejection_Or_Status</t>
         </is>
@@ -4965,6 +4965,694 @@
       <c r="U105" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1302.14 &lt;= EMA21 1304.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>224.41</v>
+      </c>
+      <c r="O106" t="n">
+        <v>229.99</v>
+      </c>
+      <c r="P106" t="n">
+        <v>229.99</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>219.16</v>
+      </c>
+      <c r="R106" t="n">
+        <v>216.86</v>
+      </c>
+      <c r="S106" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="T106" t="n">
+        <v>0</v>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 224.41 &lt;= Upper 229.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="N107" t="n">
+        <v>357.01</v>
+      </c>
+      <c r="O107" t="n">
+        <v>369.45</v>
+      </c>
+      <c r="P107" t="n">
+        <v>369.45</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>353.61</v>
+      </c>
+      <c r="R107" t="n">
+        <v>348.93</v>
+      </c>
+      <c r="S107" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="T107" t="n">
+        <v>0</v>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 357.01 &lt;= Upper 369.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>324.96</v>
+      </c>
+      <c r="O108" t="n">
+        <v>324.62</v>
+      </c>
+      <c r="P108" t="n">
+        <v>324.62</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>317.92</v>
+      </c>
+      <c r="R108" t="n">
+        <v>315.22</v>
+      </c>
+      <c r="S108" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="T108" t="n">
+        <v>0</v>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.85x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="N109" t="n">
+        <v>496.82</v>
+      </c>
+      <c r="O109" t="n">
+        <v>514.35</v>
+      </c>
+      <c r="P109" t="n">
+        <v>514.35</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>498.32</v>
+      </c>
+      <c r="R109" t="n">
+        <v>485.33</v>
+      </c>
+      <c r="S109" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="T109" t="n">
+        <v>0</v>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 496.82 &lt;= Upper 514.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="N110" t="n">
+        <v>592.85</v>
+      </c>
+      <c r="O110" t="n">
+        <v>610.46</v>
+      </c>
+      <c r="P110" t="n">
+        <v>610.46</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>575.91</v>
+      </c>
+      <c r="R110" t="n">
+        <v>577.25</v>
+      </c>
+      <c r="S110" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="T110" t="n">
+        <v>0</v>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 575.91 &lt;= EMA21 577.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="N111" t="n">
+        <v>254.98</v>
+      </c>
+      <c r="O111" t="n">
+        <v>276.69</v>
+      </c>
+      <c r="P111" t="n">
+        <v>276.69</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>259.12</v>
+      </c>
+      <c r="R111" t="n">
+        <v>259.71</v>
+      </c>
+      <c r="S111" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="T111" t="n">
+        <v>0</v>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 259.12 &lt;= EMA21 259.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="N112" t="n">
+        <v>337.12</v>
+      </c>
+      <c r="O112" t="n">
+        <v>357.04</v>
+      </c>
+      <c r="P112" t="n">
+        <v>357.04</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>341.03</v>
+      </c>
+      <c r="R112" t="n">
+        <v>344.26</v>
+      </c>
+      <c r="S112" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="T112" t="n">
+        <v>0</v>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 341.03 &lt;= EMA21 344.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="N113" t="n">
+        <v>457.06</v>
+      </c>
+      <c r="O113" t="n">
+        <v>506.53</v>
+      </c>
+      <c r="P113" t="n">
+        <v>506.53</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>468.41</v>
+      </c>
+      <c r="R113" t="n">
+        <v>477.21</v>
+      </c>
+      <c r="S113" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="T113" t="n">
+        <v>0</v>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 468.41 &lt;= EMA21 477.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="N114" t="n">
+        <v>82.73</v>
+      </c>
+      <c r="O114" t="n">
+        <v>84.45</v>
+      </c>
+      <c r="P114" t="n">
+        <v>84.45</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>80.84</v>
+      </c>
+      <c r="R114" t="n">
+        <v>78.87</v>
+      </c>
+      <c r="S114" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T114" t="n">
+        <v>0</v>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 82.73 &lt;= Upper 84.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="N115" t="n">
+        <v>169.46</v>
+      </c>
+      <c r="O115" t="n">
+        <v>189.15</v>
+      </c>
+      <c r="P115" t="n">
+        <v>189.15</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>177.82</v>
+      </c>
+      <c r="R115" t="n">
+        <v>170.64</v>
+      </c>
+      <c r="S115" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="T115" t="n">
+        <v>0</v>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.46 &lt;= Upper 189.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="N116" t="n">
+        <v>367.24</v>
+      </c>
+      <c r="O116" t="n">
+        <v>436.13</v>
+      </c>
+      <c r="P116" t="n">
+        <v>436.13</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>369.6</v>
+      </c>
+      <c r="R116" t="n">
+        <v>377.6</v>
+      </c>
+      <c r="S116" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="T116" t="n">
+        <v>0</v>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 369.60 &lt;= EMA21 377.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="N117" t="n">
+        <v>174.96</v>
+      </c>
+      <c r="O117" t="n">
+        <v>199.72</v>
+      </c>
+      <c r="P117" t="n">
+        <v>199.72</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>177.74</v>
+      </c>
+      <c r="R117" t="n">
+        <v>170.79</v>
+      </c>
+      <c r="S117" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T117" t="n">
+        <v>0</v>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.96 &lt;= Upper 199.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>234.86</v>
+      </c>
+      <c r="O118" t="n">
+        <v>291.51</v>
+      </c>
+      <c r="P118" t="n">
+        <v>291.51</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>243.36</v>
+      </c>
+      <c r="R118" t="n">
+        <v>253.29</v>
+      </c>
+      <c r="S118" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="T118" t="n">
+        <v>0</v>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 243.36 &lt;= EMA21 253.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="N119" t="n">
+        <v>76.45</v>
+      </c>
+      <c r="O119" t="n">
+        <v>81.31</v>
+      </c>
+      <c r="P119" t="n">
+        <v>81.31</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>76.92</v>
+      </c>
+      <c r="R119" t="n">
+        <v>76.16</v>
+      </c>
+      <c r="S119" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T119" t="n">
+        <v>0</v>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 76.45 &lt;= Upper 81.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>37</v>
+      </c>
+      <c r="O120" t="n">
+        <v>42.04</v>
+      </c>
+      <c r="P120" t="n">
+        <v>42.04</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="R120" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="S120" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="T120" t="n">
+        <v>0</v>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 37.00 &lt;= Upper 42.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="N121" t="n">
+        <v>169.96</v>
+      </c>
+      <c r="O121" t="n">
+        <v>170.12</v>
+      </c>
+      <c r="P121" t="n">
+        <v>170.12</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>165.72</v>
+      </c>
+      <c r="R121" t="n">
+        <v>165.03</v>
+      </c>
+      <c r="S121" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="T121" t="n">
+        <v>0</v>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.96 &lt;= Upper 170.12)</t>
         </is>
       </c>
     </row>
@@ -8499,71 +9187,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Exit_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Exit_Price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gross_PnL_Pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Net_PnL_Pct</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PnL_Amount</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Exit_Reason</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -9278,6 +9966,57 @@
         </is>
       </c>
       <c r="M18" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>376.37</v>
+      </c>
+      <c r="E19" t="n">
+        <v>359.43</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1881.85</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-4.501</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-4.551</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-85.64</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -9335,81 +10074,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Capital</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Unrealized_PnL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total_PnL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Win_Rate</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Cash_Available</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Invested_Capital</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Total_Equity</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Win_Rate_Pct</t>
         </is>
@@ -11546,6 +12285,45 @@
         <v>198907.57</v>
       </c>
       <c r="O51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10:49:12</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="n">
+        <v>-85.64</v>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="n">
+        <v>18</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="O52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11560,61 +12338,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K143"/>
+  <dimension ref="A1:K144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Expected_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fill_Price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Slippage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -16601,6 +17379,55 @@
       <c r="K143" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:49:11</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>89CC5EDBCD</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>359.43</v>
+      </c>
+      <c r="G144" t="n">
+        <v>359.43</v>
+      </c>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" t="n">
+        <v>5</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
         </is>
       </c>
     </row>
@@ -16615,104 +17442,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unrealized_PnL_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hard_SL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Highest_High</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>376.37</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1881.85</v>
-      </c>
-      <c r="F2" t="n">
-        <v>376.37</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>359.43</v>
-      </c>
-      <c r="I2" t="n">
-        <v>384.0400085449219</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
         </is>
       </c>
     </row>
@@ -16731,27 +17517,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>

</xml_diff>

<commit_message>
state: bot run 2026-09-04T10:52 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -431,61 +431,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Upper_Band</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Qualifies</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Rejection_Or_Status</t>
         </is>
@@ -1864,6 +1864,694 @@
       <c r="K33" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 168.57 &lt;= Upper 169.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>224.41</v>
+      </c>
+      <c r="E34" t="n">
+        <v>229.99</v>
+      </c>
+      <c r="F34" t="n">
+        <v>229.99</v>
+      </c>
+      <c r="G34" t="n">
+        <v>219.16</v>
+      </c>
+      <c r="H34" t="n">
+        <v>216.86</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J34" t="b">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 224.41 &lt;= Upper 229.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>357.01</v>
+      </c>
+      <c r="E35" t="n">
+        <v>369.45</v>
+      </c>
+      <c r="F35" t="n">
+        <v>369.45</v>
+      </c>
+      <c r="G35" t="n">
+        <v>353.61</v>
+      </c>
+      <c r="H35" t="n">
+        <v>348.93</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 357.01 &lt;= Upper 369.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>324.96</v>
+      </c>
+      <c r="E36" t="n">
+        <v>324.62</v>
+      </c>
+      <c r="F36" t="n">
+        <v>324.62</v>
+      </c>
+      <c r="G36" t="n">
+        <v>317.92</v>
+      </c>
+      <c r="H36" t="n">
+        <v>315.22</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J36" t="b">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.85x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>496.82</v>
+      </c>
+      <c r="E37" t="n">
+        <v>514.35</v>
+      </c>
+      <c r="F37" t="n">
+        <v>514.35</v>
+      </c>
+      <c r="G37" t="n">
+        <v>498.32</v>
+      </c>
+      <c r="H37" t="n">
+        <v>485.33</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J37" t="b">
+        <v>0</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 496.82 &lt;= Upper 514.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>592.85</v>
+      </c>
+      <c r="E38" t="n">
+        <v>610.46</v>
+      </c>
+      <c r="F38" t="n">
+        <v>610.46</v>
+      </c>
+      <c r="G38" t="n">
+        <v>575.91</v>
+      </c>
+      <c r="H38" t="n">
+        <v>577.25</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J38" t="b">
+        <v>0</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 575.91 &lt;= EMA21 577.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>254.98</v>
+      </c>
+      <c r="E39" t="n">
+        <v>276.69</v>
+      </c>
+      <c r="F39" t="n">
+        <v>276.69</v>
+      </c>
+      <c r="G39" t="n">
+        <v>259.12</v>
+      </c>
+      <c r="H39" t="n">
+        <v>259.71</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J39" t="b">
+        <v>0</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 259.12 &lt;= EMA21 259.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>337.12</v>
+      </c>
+      <c r="E40" t="n">
+        <v>357.04</v>
+      </c>
+      <c r="F40" t="n">
+        <v>357.04</v>
+      </c>
+      <c r="G40" t="n">
+        <v>341.03</v>
+      </c>
+      <c r="H40" t="n">
+        <v>344.26</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J40" t="b">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 341.03 &lt;= EMA21 344.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>457.06</v>
+      </c>
+      <c r="E41" t="n">
+        <v>506.53</v>
+      </c>
+      <c r="F41" t="n">
+        <v>506.53</v>
+      </c>
+      <c r="G41" t="n">
+        <v>468.41</v>
+      </c>
+      <c r="H41" t="n">
+        <v>477.21</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J41" t="b">
+        <v>0</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 468.41 &lt;= EMA21 477.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>82.73</v>
+      </c>
+      <c r="E42" t="n">
+        <v>84.45</v>
+      </c>
+      <c r="F42" t="n">
+        <v>84.45</v>
+      </c>
+      <c r="G42" t="n">
+        <v>80.84</v>
+      </c>
+      <c r="H42" t="n">
+        <v>78.87</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J42" t="b">
+        <v>0</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 82.73 &lt;= Upper 84.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>169.46</v>
+      </c>
+      <c r="E43" t="n">
+        <v>189.15</v>
+      </c>
+      <c r="F43" t="n">
+        <v>189.15</v>
+      </c>
+      <c r="G43" t="n">
+        <v>177.82</v>
+      </c>
+      <c r="H43" t="n">
+        <v>170.64</v>
+      </c>
+      <c r="I43" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J43" t="b">
+        <v>0</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.46 &lt;= Upper 189.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>367.24</v>
+      </c>
+      <c r="E44" t="n">
+        <v>436.13</v>
+      </c>
+      <c r="F44" t="n">
+        <v>436.13</v>
+      </c>
+      <c r="G44" t="n">
+        <v>369.6</v>
+      </c>
+      <c r="H44" t="n">
+        <v>377.6</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="J44" t="b">
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 369.60 &lt;= EMA21 377.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>174.96</v>
+      </c>
+      <c r="E45" t="n">
+        <v>199.72</v>
+      </c>
+      <c r="F45" t="n">
+        <v>199.72</v>
+      </c>
+      <c r="G45" t="n">
+        <v>177.74</v>
+      </c>
+      <c r="H45" t="n">
+        <v>170.79</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J45" t="b">
+        <v>0</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.96 &lt;= Upper 199.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>234.86</v>
+      </c>
+      <c r="E46" t="n">
+        <v>291.51</v>
+      </c>
+      <c r="F46" t="n">
+        <v>291.51</v>
+      </c>
+      <c r="G46" t="n">
+        <v>243.36</v>
+      </c>
+      <c r="H46" t="n">
+        <v>253.29</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J46" t="b">
+        <v>0</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 243.36 &lt;= EMA21 253.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>76.45</v>
+      </c>
+      <c r="E47" t="n">
+        <v>81.31</v>
+      </c>
+      <c r="F47" t="n">
+        <v>81.31</v>
+      </c>
+      <c r="G47" t="n">
+        <v>76.92</v>
+      </c>
+      <c r="H47" t="n">
+        <v>76.16</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J47" t="b">
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 76.45 &lt;= Upper 81.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>37</v>
+      </c>
+      <c r="E48" t="n">
+        <v>42.04</v>
+      </c>
+      <c r="F48" t="n">
+        <v>42.04</v>
+      </c>
+      <c r="G48" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="H48" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J48" t="b">
+        <v>0</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 37.00 &lt;= Upper 42.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>169.96</v>
+      </c>
+      <c r="E49" t="n">
+        <v>170.12</v>
+      </c>
+      <c r="F49" t="n">
+        <v>170.12</v>
+      </c>
+      <c r="G49" t="n">
+        <v>165.72</v>
+      </c>
+      <c r="H49" t="n">
+        <v>165.03</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J49" t="b">
+        <v>0</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.96 &lt;= Upper 170.12)</t>
         </is>
       </c>
     </row>
@@ -1991,104 +2679,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unrealized_PnL_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hard_SL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Highest_High</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>376.37</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1881.85</v>
-      </c>
-      <c r="F2" t="n">
-        <v>376.37</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>359.43</v>
-      </c>
-      <c r="I2" t="n">
-        <v>384.0400085449219</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
         </is>
       </c>
     </row>
@@ -2103,71 +2750,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Exit_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Exit_Price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gross_PnL_Pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Net_PnL_Pct</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PnL_Amount</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Exit_Reason</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2219,6 +2866,57 @@
         <v>2</v>
       </c>
       <c r="M2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>376.37</v>
+      </c>
+      <c r="E3" t="n">
+        <v>359.43</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1881.85</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-4.501</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-4.551</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-85.64</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -2235,61 +2933,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Expected_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fill_Price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Slippage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -2390,6 +3088,55 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-04 10:52:56</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>44F68F0F13</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>359.43</v>
+      </c>
+      <c r="G4" t="n">
+        <v>359.43</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
         </is>
       </c>
     </row>
@@ -2408,27 +3155,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -2472,51 +3219,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cash_Available</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Invested_Capital</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total_Equity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Win_Rate_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
@@ -2586,6 +3333,39 @@
       </c>
       <c r="I3" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10:52:57</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-171.28</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>